<commit_message>
refined the prompt to some extent
</commit_message>
<xml_diff>
--- a/Validated_Records_Cleaned.xlsx
+++ b/Validated_Records_Cleaned.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="82">
   <si>
     <t>ID</t>
   </si>
@@ -133,154 +133,133 @@
     <t>Book One Part One</t>
   </si>
   <si>
-    <t>Billy</t>
-  </si>
-  <si>
-    <t>Rose</t>
-  </si>
-  <si>
-    <t>Daniel</t>
-  </si>
-  <si>
-    <t>Sarah</t>
-  </si>
-  <si>
-    <t>Barbarry</t>
-  </si>
-  <si>
-    <t>Williams</t>
-  </si>
-  <si>
-    <t>Richard</t>
-  </si>
-  <si>
-    <t>Barber</t>
-  </si>
-  <si>
-    <t>Farmer</t>
-  </si>
-  <si>
-    <t>Allen</t>
+    <t>Billy Williams</t>
+  </si>
+  <si>
+    <t>Rose Richard</t>
+  </si>
+  <si>
+    <t>Daniel Barber</t>
+  </si>
+  <si>
+    <t>Sarah Farmer</t>
+  </si>
+  <si>
+    <t>Barbarry Allen</t>
   </si>
   <si>
     <t>Aurora</t>
   </si>
   <si>
-    <t>Billy Williams, 35, healthy stout man, (Richard Browne). Formerly lived with Mr. Moore of Reedy Island, Caroline, from whence he came with the 71st Regiment about 3 years ago.</t>
-  </si>
-  <si>
-    <t>Rose Richard, 20, healthy young woman, (Thomas Richard). Property of Thomas Richard, a refugee from Philadelphia.</t>
-  </si>
-  <si>
-    <t>Daniel Barber, 70, worn out, (James Moore). Says he was made free by Mr. Austin Moore of little York nigh 20 years ago.</t>
-  </si>
-  <si>
-    <t>Sarah Farmer, 23, healthy young woman, (Mrs. Sharp).</t>
-  </si>
-  <si>
-    <t>Barbarry Allen, 22, healthy stout wench, (Humphry Winters). Property of Humphrey Winters of New York from Virginia.</t>
+    <t>20</t>
   </si>
   <si>
     <t>Ship Aurora bound for St. John's</t>
   </si>
   <si>
-    <t>Ship Aurora bound for St. John's</t>
+    <t>African American</t>
+  </si>
+  <si>
+    <t>Property of Humphrey Winters of New York from Virginia</t>
+  </si>
+  <si>
+    <t>17</t>
+  </si>
+  <si>
+    <t>Black</t>
+  </si>
+  <si>
+    <t>Book of Negroes, British Headquarters Papers PRO 30/55/100; Loyalist evacuation shipping lists (1782–1784)</t>
+  </si>
+  <si>
+    <t>Female</t>
+  </si>
+  <si>
+    <t>-</t>
   </si>
   <si>
     <t>1748</t>
   </si>
   <si>
-    <t>1763</t>
-  </si>
-  <si>
-    <t>1913</t>
-  </si>
-  <si>
-    <t>1760</t>
+    <t>Male</t>
+  </si>
+  <si>
+    <t>Philadelphia</t>
+  </si>
+  <si>
+    <t>Princess Ann</t>
+  </si>
+  <si>
+    <t>Virginia</t>
+  </si>
+  <si>
+    <t>United States</t>
+  </si>
+  <si>
+    <t>little York</t>
+  </si>
+  <si>
+    <t>Reedy Island</t>
+  </si>
+  <si>
+    <t>St. John's</t>
+  </si>
+  <si>
+    <t>New York</t>
+  </si>
+  <si>
+    <t>Caroline</t>
+  </si>
+  <si>
+    <t>39.9527237, -75.1635262</t>
+  </si>
+  <si>
+    <t>1783</t>
+  </si>
+  <si>
+    <t>Canada</t>
+  </si>
+  <si>
+    <t>47.5646794, -52.7066964</t>
+  </si>
+  <si>
+    <t>MRS. SHARP</t>
+  </si>
+  <si>
+    <t>Thomas Richard</t>
+  </si>
+  <si>
+    <t>James Moore</t>
+  </si>
+  <si>
+    <t>Father_FirstName: -</t>
+  </si>
+  <si>
+    <t>Humphry Winters</t>
+  </si>
+  <si>
+    <t>Richard Browne</t>
+  </si>
+  <si>
+    <t>Father_Surname: -</t>
+  </si>
+  <si>
+    <t>1713</t>
+  </si>
+  <si>
+    <t>Mother_FirstName: -</t>
+  </si>
+  <si>
+    <t>41.0111483, -90.7462496</t>
+  </si>
+  <si>
+    <t>Mother_Surname: -</t>
   </si>
   <si>
     <t>1761</t>
   </si>
   <si>
-    <t>Male</t>
-  </si>
-  <si>
-    <t>Female</t>
-  </si>
-  <si>
-    <t>Black</t>
-  </si>
-  <si>
-    <t>African American</t>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>Philadelphia</t>
-  </si>
-  <si>
-    <t>little York</t>
-  </si>
-  <si>
-    <t>Caroline</t>
-  </si>
-  <si>
-    <t>Virginia</t>
-  </si>
-  <si>
-    <t>Reedy Island</t>
-  </si>
-  <si>
-    <t>United States</t>
-  </si>
-  <si>
-    <t>37.5329655, -77.471394</t>
-  </si>
-  <si>
-    <t>39.9527237, -75.1635262</t>
-  </si>
-  <si>
-    <t>41.0111483, -90.7462496</t>
-  </si>
-  <si>
-    <t>New York</t>
-  </si>
-  <si>
-    <t>40.7128, -74.0060</t>
-  </si>
-  <si>
-    <t>1783</t>
-  </si>
-  <si>
-    <t>St. John's</t>
-  </si>
-  <si>
-    <t>Canada</t>
-  </si>
-  <si>
-    <t>45.2733, -66.0633</t>
-  </si>
-  <si>
-    <t>17</t>
-  </si>
-  <si>
-    <t>James Moore</t>
-  </si>
-  <si>
-    <t>Humphry Winters</t>
-  </si>
-  <si>
-    <t>Richard Browne</t>
-  </si>
-  <si>
-    <t>Thomas Richard</t>
-  </si>
-  <si>
-    <t>Book of Negroes, British Headquarters Papers PRO 30/55/100; Loyalist evacuation shipping lists (1782–1784)</t>
-  </si>
-  <si>
-    <t>Mrs. Sharp</t>
+    <t>Mixed Race</t>
   </si>
 </sst>
 </file>
@@ -730,91 +709,91 @@
         <v>44</v>
       </c>
       <c r="E2" t="s">
+        <v>46</v>
+      </c>
+      <c r="F2" t="s">
         <v>49</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
+        <v>51</v>
+      </c>
+      <c r="H2" t="s">
+        <v>53</v>
+      </c>
+      <c r="I2" t="s">
+        <v>54</v>
+      </c>
+      <c r="J2" t="s">
+        <v>55</v>
+      </c>
+      <c r="K2" t="s">
         <v>50</v>
       </c>
-      <c r="G2" t="s">
-        <v>55</v>
-      </c>
-      <c r="H2" t="s">
-        <v>57</v>
-      </c>
-      <c r="I2" t="s">
+      <c r="L2" t="s">
+        <v>47</v>
+      </c>
+      <c r="M2" t="s">
+        <v>50</v>
+      </c>
+      <c r="N2" t="s">
+        <v>61</v>
+      </c>
+      <c r="O2" t="s">
+        <v>64</v>
+      </c>
+      <c r="P2" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>59</v>
+      </c>
+      <c r="R2" t="s">
+        <v>63</v>
+      </c>
+      <c r="S2" t="s">
+        <v>63</v>
+      </c>
+      <c r="T2" t="s">
+        <v>66</v>
+      </c>
+      <c r="U2" t="s">
         <v>62</v>
       </c>
-      <c r="J2" t="s">
-        <v>64</v>
-      </c>
-      <c r="K2" t="s">
-        <v>65</v>
-      </c>
-      <c r="L2" t="s">
-        <v>66</v>
-      </c>
-      <c r="M2" t="s">
-        <v>66</v>
-      </c>
-      <c r="N2" t="s">
-        <v>69</v>
-      </c>
-      <c r="O2" t="s">
-        <v>71</v>
-      </c>
-      <c r="P2" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>66</v>
-      </c>
-      <c r="R2" t="s">
-        <v>66</v>
-      </c>
-      <c r="S2" t="s">
-        <v>77</v>
-      </c>
-      <c r="T2" t="s">
-        <v>76</v>
-      </c>
-      <c r="U2" t="s">
-        <v>76</v>
-      </c>
       <c r="V2" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="W2" t="s">
-        <v>79</v>
+        <v>68</v>
       </c>
       <c r="X2" t="s">
-        <v>80</v>
+        <v>62</v>
       </c>
       <c r="Y2" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="Z2" t="s">
-        <v>66</v>
+        <v>53</v>
       </c>
       <c r="AA2" t="s">
-        <v>66</v>
+        <v>53</v>
       </c>
       <c r="AB2" t="s">
-        <v>66</v>
+        <v>53</v>
       </c>
       <c r="AC2" t="s">
-        <v>66</v>
+        <v>53</v>
       </c>
       <c r="AD2" t="s">
-        <v>82</v>
+        <v>53</v>
       </c>
       <c r="AE2" t="s">
-        <v>79</v>
+        <v>53</v>
       </c>
       <c r="AF2" t="s">
-        <v>85</v>
+        <v>53</v>
       </c>
       <c r="AG2" t="s">
-        <v>87</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:33">
@@ -831,91 +810,91 @@
         <v>45</v>
       </c>
       <c r="E3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F3" t="s">
+        <v>50</v>
+      </c>
+      <c r="G3" t="s">
+        <v>52</v>
+      </c>
+      <c r="H3" t="s">
+        <v>53</v>
+      </c>
+      <c r="I3" t="s">
+        <v>50</v>
+      </c>
+      <c r="J3" t="s">
+        <v>56</v>
+      </c>
+      <c r="K3" t="s">
+        <v>57</v>
+      </c>
+      <c r="L3" t="s">
+        <v>58</v>
+      </c>
+      <c r="M3" t="s">
+        <v>59</v>
+      </c>
+      <c r="N3" t="s">
+        <v>53</v>
+      </c>
+      <c r="O3" t="s">
+        <v>53</v>
+      </c>
+      <c r="P3" t="s">
+        <v>59</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>65</v>
+      </c>
+      <c r="R3" t="s">
+        <v>63</v>
+      </c>
+      <c r="S3" t="s">
+        <v>63</v>
+      </c>
+      <c r="T3" t="s">
+        <v>66</v>
+      </c>
+      <c r="U3" t="s">
+        <v>62</v>
+      </c>
+      <c r="V3" t="s">
+        <v>67</v>
+      </c>
+      <c r="W3" t="s">
+        <v>53</v>
+      </c>
+      <c r="X3" t="s">
+        <v>70</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>62</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>70</v>
+      </c>
+      <c r="AA3" t="s">
         <v>51</v>
       </c>
-      <c r="G3" t="s">
-        <v>56</v>
-      </c>
-      <c r="H3" t="s">
-        <v>58</v>
-      </c>
-      <c r="I3" t="s">
-        <v>63</v>
-      </c>
-      <c r="J3" t="s">
-        <v>64</v>
-      </c>
-      <c r="K3" t="s">
-        <v>65</v>
-      </c>
-      <c r="L3" t="s">
-        <v>66</v>
-      </c>
-      <c r="M3" t="s">
-        <v>67</v>
-      </c>
-      <c r="N3" t="s">
-        <v>66</v>
-      </c>
-      <c r="O3" t="s">
-        <v>66</v>
-      </c>
-      <c r="P3" t="s">
-        <v>66</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>72</v>
-      </c>
-      <c r="R3" t="s">
-        <v>74</v>
-      </c>
-      <c r="S3" t="s">
-        <v>76</v>
-      </c>
-      <c r="T3" t="s">
-        <v>76</v>
-      </c>
-      <c r="U3" t="s">
-        <v>78</v>
-      </c>
-      <c r="V3" t="s">
-        <v>79</v>
-      </c>
-      <c r="W3" t="s">
-        <v>80</v>
-      </c>
-      <c r="X3" t="s">
-        <v>66</v>
-      </c>
-      <c r="Y3" t="s">
-        <v>66</v>
-      </c>
-      <c r="Z3" t="s">
-        <v>66</v>
-      </c>
-      <c r="AA3" t="s">
-        <v>66</v>
-      </c>
       <c r="AB3" t="s">
-        <v>66</v>
+        <v>53</v>
       </c>
       <c r="AC3" t="s">
-        <v>66</v>
+        <v>53</v>
       </c>
       <c r="AD3" t="s">
-        <v>82</v>
+        <v>53</v>
       </c>
       <c r="AE3" t="s">
-        <v>79</v>
+        <v>53</v>
       </c>
       <c r="AF3" t="s">
-        <v>86</v>
+        <v>53</v>
       </c>
       <c r="AG3" t="s">
-        <v>87</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4" spans="1:33">
@@ -929,94 +908,94 @@
         <v>41</v>
       </c>
       <c r="D4" t="s">
+        <v>44</v>
+      </c>
+      <c r="E4" t="s">
         <v>46</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>49</v>
       </c>
-      <c r="F4" t="s">
-        <v>52</v>
-      </c>
       <c r="G4" t="s">
+        <v>51</v>
+      </c>
+      <c r="H4" t="s">
+        <v>53</v>
+      </c>
+      <c r="I4" t="s">
         <v>55</v>
       </c>
-      <c r="H4" t="s">
+      <c r="J4" t="s">
+        <v>50</v>
+      </c>
+      <c r="K4" t="s">
+        <v>47</v>
+      </c>
+      <c r="L4" t="s">
+        <v>53</v>
+      </c>
+      <c r="M4" t="s">
+        <v>60</v>
+      </c>
+      <c r="N4" t="s">
+        <v>53</v>
+      </c>
+      <c r="O4" t="s">
+        <v>53</v>
+      </c>
+      <c r="P4" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q4" t="s">
         <v>59</v>
       </c>
-      <c r="I4" t="s">
+      <c r="R4" t="s">
+        <v>63</v>
+      </c>
+      <c r="S4" t="s">
+        <v>66</v>
+      </c>
+      <c r="T4" t="s">
         <v>62</v>
       </c>
-      <c r="J4" t="s">
-        <v>64</v>
-      </c>
-      <c r="K4" t="s">
-        <v>65</v>
-      </c>
-      <c r="L4" t="s">
+      <c r="U4" t="s">
+        <v>67</v>
+      </c>
+      <c r="V4" t="s">
+        <v>53</v>
+      </c>
+      <c r="W4" t="s">
+        <v>62</v>
+      </c>
+      <c r="X4" t="s">
+        <v>71</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>53</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>76</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>78</v>
+      </c>
+      <c r="AB4" t="s">
+        <v>63</v>
+      </c>
+      <c r="AC4" t="s">
         <v>66</v>
       </c>
-      <c r="M4" t="s">
-        <v>68</v>
-      </c>
-      <c r="N4" t="s">
+      <c r="AD4" t="s">
+        <v>63</v>
+      </c>
+      <c r="AE4" t="s">
         <v>66</v>
       </c>
-      <c r="O4" t="s">
-        <v>66</v>
-      </c>
-      <c r="P4" t="s">
-        <v>66</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>72</v>
-      </c>
-      <c r="R4" t="s">
-        <v>75</v>
-      </c>
-      <c r="S4" t="s">
-        <v>76</v>
-      </c>
-      <c r="T4" t="s">
-        <v>76</v>
-      </c>
-      <c r="U4" t="s">
-        <v>78</v>
-      </c>
-      <c r="V4" t="s">
-        <v>79</v>
-      </c>
-      <c r="W4" t="s">
-        <v>80</v>
-      </c>
-      <c r="X4" t="s">
-        <v>66</v>
-      </c>
-      <c r="Y4" t="s">
-        <v>66</v>
-      </c>
-      <c r="Z4" t="s">
-        <v>66</v>
-      </c>
-      <c r="AA4" t="s">
-        <v>66</v>
-      </c>
-      <c r="AB4" t="s">
-        <v>66</v>
-      </c>
-      <c r="AC4" t="s">
-        <v>82</v>
-      </c>
-      <c r="AD4" t="s">
-        <v>79</v>
-      </c>
-      <c r="AE4" t="s">
-        <v>83</v>
-      </c>
       <c r="AF4" t="s">
-        <v>87</v>
+        <v>62</v>
       </c>
       <c r="AG4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="5" spans="1:33">
@@ -1030,94 +1009,94 @@
         <v>42</v>
       </c>
       <c r="D5" t="s">
+        <v>44</v>
+      </c>
+      <c r="E5" t="s">
+        <v>46</v>
+      </c>
+      <c r="F5" t="s">
+        <v>49</v>
+      </c>
+      <c r="G5" t="s">
+        <v>51</v>
+      </c>
+      <c r="H5" t="s">
+        <v>53</v>
+      </c>
+      <c r="I5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J5" t="s">
+        <v>50</v>
+      </c>
+      <c r="K5" t="s">
         <v>47</v>
       </c>
-      <c r="E5" t="s">
+      <c r="L5" t="s">
+        <v>50</v>
+      </c>
+      <c r="M5" t="s">
+        <v>53</v>
+      </c>
+      <c r="N5" t="s">
+        <v>62</v>
+      </c>
+      <c r="O5" t="s">
+        <v>59</v>
+      </c>
+      <c r="P5" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>66</v>
+      </c>
+      <c r="R5" t="s">
+        <v>62</v>
+      </c>
+      <c r="S5" t="s">
+        <v>67</v>
+      </c>
+      <c r="T5" t="s">
+        <v>68</v>
+      </c>
+      <c r="U5" t="s">
+        <v>62</v>
+      </c>
+      <c r="V5" t="s">
+        <v>69</v>
+      </c>
+      <c r="W5" t="s">
+        <v>53</v>
+      </c>
+      <c r="X5" t="s">
+        <v>72</v>
+      </c>
+      <c r="Y5" t="s">
+        <v>75</v>
+      </c>
+      <c r="Z5" t="s">
+        <v>77</v>
+      </c>
+      <c r="AA5" t="s">
+        <v>79</v>
+      </c>
+      <c r="AB5" t="s">
         <v>49</v>
       </c>
-      <c r="F5" t="s">
-        <v>53</v>
-      </c>
-      <c r="G5" t="s">
-        <v>56</v>
-      </c>
-      <c r="H5" t="s">
-        <v>60</v>
-      </c>
-      <c r="I5" t="s">
-        <v>63</v>
-      </c>
-      <c r="J5" t="s">
-        <v>64</v>
-      </c>
-      <c r="K5" t="s">
-        <v>65</v>
-      </c>
-      <c r="L5" t="s">
-        <v>66</v>
-      </c>
-      <c r="M5" t="s">
-        <v>66</v>
-      </c>
-      <c r="N5" t="s">
-        <v>66</v>
-      </c>
-      <c r="O5" t="s">
-        <v>66</v>
-      </c>
-      <c r="P5" t="s">
-        <v>66</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>72</v>
-      </c>
-      <c r="R5" t="s">
-        <v>66</v>
-      </c>
-      <c r="S5" t="s">
-        <v>66</v>
-      </c>
-      <c r="T5" t="s">
-        <v>66</v>
-      </c>
-      <c r="U5" t="s">
-        <v>66</v>
-      </c>
-      <c r="V5" t="s">
-        <v>66</v>
-      </c>
-      <c r="W5" t="s">
-        <v>78</v>
-      </c>
-      <c r="X5" t="s">
-        <v>79</v>
-      </c>
-      <c r="Y5" t="s">
-        <v>80</v>
-      </c>
-      <c r="Z5" t="s">
-        <v>66</v>
-      </c>
-      <c r="AA5" t="s">
-        <v>66</v>
-      </c>
-      <c r="AB5" t="s">
-        <v>66</v>
-      </c>
       <c r="AC5" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="AD5" t="s">
-        <v>82</v>
+        <v>69</v>
       </c>
       <c r="AE5" t="s">
-        <v>66</v>
+        <v>51</v>
       </c>
       <c r="AF5" t="s">
-        <v>88</v>
+        <v>53</v>
       </c>
       <c r="AG5" t="s">
-        <v>87</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6" spans="1:33">
@@ -1131,94 +1110,94 @@
         <v>43</v>
       </c>
       <c r="D6" t="s">
+        <v>44</v>
+      </c>
+      <c r="E6" t="s">
         <v>48</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
+        <v>46</v>
+      </c>
+      <c r="G6" t="s">
         <v>49</v>
       </c>
-      <c r="F6" t="s">
-        <v>54</v>
-      </c>
-      <c r="G6" t="s">
-        <v>56</v>
-      </c>
-      <c r="H6" t="s">
-        <v>61</v>
+      <c r="H6">
+        <v>1753</v>
       </c>
       <c r="I6" t="s">
+        <v>53</v>
+      </c>
+      <c r="J6" t="s">
+        <v>52</v>
+      </c>
+      <c r="K6" t="s">
+        <v>50</v>
+      </c>
+      <c r="L6" t="s">
+        <v>47</v>
+      </c>
+      <c r="M6" t="s">
+        <v>53</v>
+      </c>
+      <c r="N6" t="s">
         <v>63</v>
       </c>
-      <c r="J6" t="s">
-        <v>64</v>
-      </c>
-      <c r="K6" t="s">
-        <v>65</v>
-      </c>
-      <c r="L6" t="s">
+      <c r="O6" t="s">
+        <v>53</v>
+      </c>
+      <c r="P6" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>53</v>
+      </c>
+      <c r="R6" t="s">
+        <v>59</v>
+      </c>
+      <c r="S6" t="s">
+        <v>63</v>
+      </c>
+      <c r="T6" t="s">
         <v>66</v>
       </c>
-      <c r="M6" t="s">
-        <v>66</v>
-      </c>
-      <c r="N6" t="s">
-        <v>70</v>
-      </c>
-      <c r="O6" t="s">
-        <v>66</v>
-      </c>
-      <c r="P6" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q6" t="s">
+      <c r="U6" t="s">
+        <v>62</v>
+      </c>
+      <c r="V6" t="s">
+        <v>67</v>
+      </c>
+      <c r="W6" t="s">
+        <v>53</v>
+      </c>
+      <c r="X6" t="s">
         <v>73</v>
       </c>
-      <c r="R6" t="s">
-        <v>76</v>
-      </c>
-      <c r="S6" t="s">
-        <v>76</v>
-      </c>
-      <c r="T6" t="s">
-        <v>78</v>
-      </c>
-      <c r="U6" t="s">
-        <v>79</v>
-      </c>
-      <c r="V6" t="s">
+      <c r="Y6" t="s">
+        <v>62</v>
+      </c>
+      <c r="Z6" t="s">
+        <v>43</v>
+      </c>
+      <c r="AA6" t="s">
         <v>80</v>
       </c>
-      <c r="W6" t="s">
-        <v>66</v>
-      </c>
-      <c r="X6" t="s">
-        <v>66</v>
-      </c>
-      <c r="Y6" t="s">
-        <v>66</v>
-      </c>
-      <c r="Z6" t="s">
-        <v>66</v>
-      </c>
-      <c r="AA6" t="s">
-        <v>66</v>
-      </c>
       <c r="AB6" t="s">
-        <v>66</v>
+        <v>50</v>
       </c>
       <c r="AC6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AD6" t="s">
-        <v>79</v>
+        <v>53</v>
       </c>
       <c r="AE6" t="s">
-        <v>84</v>
+        <v>59</v>
       </c>
       <c r="AF6" t="s">
-        <v>87</v>
+        <v>53</v>
       </c>
       <c r="AG6" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
   </sheetData>

</xml_diff>